<commit_message>
updated ULI calculation and related dashboard visualisation and prose output, along with option to calculate walkability variants (eg attenuated by thermal comfort)
</commit_message>
<xml_diff>
--- a/process/configuration/assets/output_data_dictionary.xlsx
+++ b/process/configuration/assets/output_data_dictionary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F111"/>
+  <dimension ref="A1:F129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2091,22 +2091,22 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (straight-line catchment)</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Average population density of the local walkable neighbourhood (population per km², based on the population grid cells intersecting the sample point neighbourhood)</t>
+          <t>Straight-line distance (m) to the nearest destination, missing beyond the distance searched (max_distance)</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>sp_local_nh_avg_pop_density</t>
+          <t>sp_euclid_dist_[destination]</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>persons per km²</t>
+          <t>metres</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -2123,22 +2123,22 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (straight-line catchment)</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Average street intersection density of the local walkable neighbourhood (intersections per km²)</t>
+          <t>Score (0/1): the destination lies within [x] m in a straight line</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>sp_local_nh_avg_intersection_density</t>
+          <t>sp_euclid_access_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>count per km²</t>
+          <t>score 0-1</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
@@ -2155,22 +2155,22 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (straight-line catchment)</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Daily living score (/3): sum of access scores for fresh food, convenience and public transport destinations</t>
+          <t>Score (0/1): the nearest destination (a disamenity) is further than [x] m in a straight line</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>sp_daily_living_score</t>
+          <t>sp_euclid_beyond_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>score 0-3</t>
+          <t>score 0-1</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -2187,118 +2187,118 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (straight-line catchment)</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Walkability index: sum of z-scores of the daily living score, neighbourhood population density and neighbourhood intersection density</t>
+          <t>Percentage of population within [x] m in a straight line of the destination</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>sp_walkability_index</t>
+          <t>pct_access_euclid_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>index (sum of z-scores)</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>percentage</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (straight-line catchment)</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood population density (population per km²) of sample points in this area</t>
+          <t>Percentage of population within [x] m in a straight line of the destination (population weighted)</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>local_nh_population_density</t>
+          <t>pop_pct_access_euclid_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>persons per km²</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>percentage</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>grid, city, custom areas</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (straight-line catchment)</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood intersection density (intersections per km²) of sample points in this area</t>
+          <t>Percentage of population living further than [x] m in a straight line from the nearest destination (a disamenity)</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>local_nh_intersection_density</t>
+          <t>pct_beyond_euclid_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>count per km²</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>percentage</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>grid, city, custom areas</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (straight-line catchment)</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Average daily living score (/3) of sample points in this area</t>
+          <t>Average straight-line distance (m) to the nearest destination</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>local_daily_living</t>
+          <t>avg_euclid_dist_[destination]</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>score 0-3</t>
+          <t>metres</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2308,29 +2308,29 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>grid, city, custom areas</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Indicator estimates: walkability</t>
+          <t>Indicator estimates: access (straight-line catchment)</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Average walkability index of sample points in this area</t>
+          <t>Average straight-line distance (m) to the nearest destination (population weighted)</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>local_walkability</t>
+          <t>pop_avg_euclid_dist_[destination]</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>index (sum of z-scores)</t>
+          <t>metres</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2340,7 +2340,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>grid, city, custom areas</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
@@ -2352,12 +2352,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood population density (population per km²; population weighted)</t>
+          <t>Average population density of the local walkable neighbourhood (population per km², based on the population grid cells intersecting the sample point neighbourhood)</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>pop_nh_pop_density</t>
+          <t>sp_local_nh_avg_pop_density</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2367,12 +2367,12 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
@@ -2384,12 +2384,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Average walkable neighbourhood intersection density (intersections per km²; population weighted)</t>
+          <t>Average street intersection density of the local walkable neighbourhood (intersections per km²)</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>pop_nh_intersection_density</t>
+          <t>sp_local_nh_avg_intersection_density</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -2399,12 +2399,12 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
@@ -2416,12 +2416,12 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Average daily living score (/3; population weighted)</t>
+          <t>Daily living score (/3): sum of access scores for fresh food, convenience and public transport destinations</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>pop_daily_living</t>
+          <t>sp_daily_living_score</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2431,12 +2431,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
@@ -2448,12 +2448,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Average walkability index (population weighted)</t>
+          <t>Walkability index: sum of z-scores of the daily living score, neighbourhood population density and neighbourhood intersection density</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>pop_walkability</t>
+          <t>sp_walkability_index</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2463,162 +2463,162 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Score (0/1): the destination is reachable within [x] m by cycling, routed using the [network] measure</t>
+          <t>Average walkable neighbourhood population density (population per km²) of sample points in this area</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>sp_cycle_[network]access_[destination]_[x]m</t>
+          <t>local_nh_population_density</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>score 0-1</t>
+          <t>persons per km²</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Distance (m) by cycling to the nearest destination, routed using the [network] measure</t>
+          <t>Average walkable neighbourhood intersection density (intersections per km²) of sample points in this area</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>sp_cycle_[network]nearest_node_[destination]</t>
+          <t>local_nh_intersection_density</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>metres</t>
+          <t>count per km²</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>sample point</t>
+          <t>grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Percentage of population with cycling access within [x] m to the destination, routed using the [network] measure</t>
+          <t>Average daily living score (/3) of sample points in this area</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>pct_access_cycle_[network][destination]_[x]m</t>
+          <t>local_daily_living</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>score 0-3</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>percentage</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>grid, custom areas</t>
+          <t>grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Percentage of population with cycling access within [x] m to the destination, routed using the [network] measure (population weighted)</t>
+          <t>Average walkability index of sample points in this area</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>pop_pct_access_cycle_[network][destination]_[x]m</t>
+          <t>local_walkability</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>index (sum of z-scores)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>percentage</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>city, custom areas</t>
+          <t>grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Average distance (m) by cycling to the nearest destination, routed using the [network] measure</t>
+          <t>Average walkable neighbourhood population density (population per km²; population weighted)</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>avg_cycle_dist_[network][destination]</t>
+          <t>pop_nh_pop_density</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>metres</t>
+          <t>persons per km²</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -2628,29 +2628,29 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>grid, custom areas</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Indicator estimates: cycling accessibility</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Average distance (m) by cycling to the nearest destination, routed using the [network] measure (population weighted)</t>
+          <t>Average walkable neighbourhood intersection density (intersections per km²; population weighted)</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>pop_avg_cycle_dist_[network][destination]</t>
+          <t>pop_nh_intersection_density</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>metres</t>
+          <t>count per km²</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -2667,22 +2667,22 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Heat Exposure Index (HEI): the heat exposure sub-index, derived from land surface temperature</t>
+          <t>Average daily living score (/3; population weighted)</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>urban_heat_exposure_index</t>
+          <t>pop_daily_living</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>index 0-100</t>
+          <t>score 0-3</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -2692,29 +2692,29 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: walkability</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Land surface temperature (°C): the temperature of the Earth’s surface, indicating the lived experience of heat (Landsat 8 surface reflectance, hottest third of the year)</t>
+          <t>Average walkability index (population weighted)</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>urban_heat_land_surface_temp_c</t>
+          <t>pop_walkability</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>degrees Celsius</t>
+          <t>index (sum of z-scores)</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
@@ -2724,189 +2724,189 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Heat Sensitivity Index (HSI): the equally weighted heat sensitivity sub-index of land surface albedo, NDVI, NDBI, local climate zone, population density and vulnerable population</t>
+          <t>Score (0/1): the destination is reachable within [x] m by cycling, routed using the [network] measure</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>urban_heat_sensitivity_index</t>
+          <t>sp_cycle_[network]access_[destination]_[x]m</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>index 0-100</t>
+          <t>score 0-1</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Land surface albedo: solar reflectance, where higher reflectance implies less surface heat retention (inverted, so that higher values indicate greater heat vulnerability)</t>
+          <t>Distance (m) by cycling to the nearest destination, routed using the [network] measure</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>urban_heat_land_surface_albedo</t>
+          <t>sp_cycle_[network]nearest_node_[destination]</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>proportion 0-1</t>
+          <t>metres</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>value</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Normalised Difference Vegetation Index (NDVI): a spectral index of vegetation health and greenness (inverted, so that higher values indicate greater heat vulnerability)</t>
+          <t>Percentage of population with cycling access within [x] m to the destination, routed using the [network] measure</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>urban_heat_ndvi</t>
+          <t>pct_access_cycle_[network][destination]_[x]m</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>index -1 to 1</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>percentage</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Normalised Difference Built-up Index (NDBI): a spectral index of impervious surfaces such as concrete and asphalt</t>
+          <t>Percentage of population with cycling access within [x] m to the destination, routed using the [network] measure (population weighted)</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>urban_heat_ndbi</t>
+          <t>pop_pct_access_cycle_[network][destination]_[x]m</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>index -1 to 1</t>
+          <t>percent</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>mean</t>
+          <t>percentage</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Local Climate Zone: a standardised classification of land cover typologies for urban heat island studies, ordered from least heat retaining (water) to most heat retaining (bare rock or paved)</t>
+          <t>Average distance (m) by cycling to the nearest destination, routed using the [network] measure</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>urban_heat_local_climate_zone_ordered</t>
+          <t>avg_cycle_dist_[network][destination]</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>ordered class</t>
+          <t>metres</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>category</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Indicator estimates: urban heat vulnerability</t>
+          <t>Indicator estimates: cycling accessibility</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Population density (persons per km²), from the GHS-POP global human settlement population grid</t>
+          <t>Average distance (m) by cycling to the nearest destination, routed using the [network] measure (population weighted)</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>urban_heat_population_density_per_sqkm</t>
+          <t>pop_avg_cycle_dist_[network][destination]</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>persons per km²</t>
+          <t>metres</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -2916,7 +2916,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>sample point, grid, city, custom areas</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
@@ -2928,22 +2928,22 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Vulnerable population (%): those most at risk from heat on the basis of age, being the combined proportion of the population aged 0–4 and 65+ years</t>
+          <t>Heat Exposure Index (HEI): the heat exposure sub-index, derived from land surface temperature</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>urban_heat_vulnerable_pop_pct</t>
+          <t>urban_heat_exposure_index</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>index 0-100</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>percentage</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
@@ -2960,17 +2960,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Adaptive Capability Index (ACI): the equally weighted adaptive capability sub-index of child dependency ratio, subnational Human Development Index and infant mortality rate; higher values indicate lower adaptive capability</t>
+          <t>Land surface temperature (°C): the temperature of the Earth’s surface, indicating the lived experience of heat (Landsat 8 surface reflectance, hottest third of the year)</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>urban_heat_adaptive_capability_index</t>
+          <t>urban_heat_land_surface_temp_c</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>index 0-100</t>
+          <t>degrees Celsius</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
@@ -2992,17 +2992,17 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Child dependency ratio: children (aged 0–14 years) relative to the working age population (15–64 years), indicating economic reliance</t>
+          <t>Heat Sensitivity Index (HSI): the equally weighted heat sensitivity sub-index of land surface albedo, NDVI, NDBI, local climate zone, population density and vulnerable population</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>urban_heat_child_dependency_ratio</t>
+          <t>urban_heat_sensitivity_index</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>ratio</t>
+          <t>index 0-100</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -3024,17 +3024,17 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Subnational Human Development Index: human well-being assessed through education, health and standard of living</t>
+          <t>Land surface albedo: solar reflectance, where higher reflectance implies less surface heat retention (inverted, so that higher values indicate greater heat vulnerability)</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>urban_heat_subnational_hdi</t>
+          <t>urban_heat_land_surface_albedo</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>index 0-100</t>
+          <t>proportion 0-1</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
@@ -3056,17 +3056,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Infant mortality rate: deaths of children under 1 year of age per 1000 live births, a key indicator of population health</t>
+          <t>Normalised Difference Vegetation Index (NDVI): a spectral index of vegetation health and greenness (inverted, so that higher values indicate greater heat vulnerability)</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>urban_heat_infant_mortality_rate</t>
+          <t>urban_heat_ndvi</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>deaths per 1,000 live births</t>
+          <t>index -1 to 1</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -3088,17 +3088,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Global Urban Heat Vulnerability Index (GUHVI): the equally weighted composite of the Heat Exposure, Heat Sensitivity and Adaptive Capability indices, (HEI + HSI + ACI) / 3</t>
+          <t>Normalised Difference Built-up Index (NDBI): a spectral index of impervious surfaces such as concrete and asphalt</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>urban_heat_guhvi</t>
+          <t>urban_heat_ndbi</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>index 0-100</t>
+          <t>index -1 to 1</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -3120,17 +3120,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Global Urban Heat Vulnerability Index (GUHVI) class, from 1 (least vulnerable) to 5 (most vulnerable)</t>
+          <t>Local Climate Zone: a standardised classification of land cover typologies for urban heat island studies, ordered from least heat retaining (water) to most heat retaining (bare rock or paved)</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>urban_heat_guhvi_class</t>
+          <t>urban_heat_local_climate_zone_ordered</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>class 1-5</t>
+          <t>ordered class</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
@@ -3152,459 +3152,603 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Percentage of population in Global Urban Heat Vulnerability Index (GUHVI) class 5, the most vulnerable class</t>
+          <t>Population density (persons per km²), from the GHS-POP global human settlement population grid</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>pct_urban_heat_guhvi_class_5_most_vulnerable</t>
+          <t>urban_heat_population_density_per_sqkm</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>percent</t>
+          <t>persons per km²</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>percentage</t>
+          <t>mean</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>grid, city, custom areas</t>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Timepoint label of the observation (e.g. year)</t>
+          <t>Vulnerable population (%): those most at risk from heat on the basis of age, being the combined proportion of the population aged 0–4 and 65+ years</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>timepoint</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr"/>
-      <c r="E93" t="inlineStr"/>
+          <t>urban_heat_vulnerable_pop_pct</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Output variable name of the indicator observed (see the indicator entries of this data dictionary)</t>
+          <t>Adaptive Capability Index (ACI): the equally weighted adaptive capability sub-index of child dependency ratio, subnational Human Development Index and infant mortality rate; higher values indicate lower adaptive capability</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>indicator</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr"/>
-      <c r="E94" t="inlineStr"/>
+          <t>urban_heat_adaptive_capability_index</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>index 0-100</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Value of the indicator at this timepoint for this unit</t>
+          <t>Child dependency ratio: children (aged 0–14 years) relative to the working age population (15–64 years), indicating economic reliance</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr"/>
-      <c r="E95" t="inlineStr"/>
+          <t>urban_heat_child_dependency_ratio</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>ratio</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Custom area identifier (area panels)</t>
+          <t>Subnational Human Development Index: human well-being assessed through education, health and standard of living</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>area_id</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr"/>
-      <c r="E96" t="inlineStr"/>
+          <t>urban_heat_subnational_hdi</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>index 0-100</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Unit identifier (generic panels)</t>
+          <t>Infant mortality rate: deaths of children under 1 year of age per 1000 live births, a key indicator of population health</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>unit_id</t>
-        </is>
-      </c>
-      <c r="D97" t="inlineStr"/>
-      <c r="E97" t="inlineStr"/>
+          <t>urban_heat_infant_mortality_rate</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>deaths per 1,000 live births</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Baseline timepoint label of the comparison pair</t>
+          <t>Global Urban Heat Vulnerability Index (GUHVI): the equally weighted composite of the Heat Exposure, Heat Sensitivity and Adaptive Capability indices, (HEI + HSI + ACI) / 3</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>t0</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr"/>
-      <c r="E98" t="inlineStr"/>
+          <t>urban_heat_guhvi</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>index 0-100</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Follow-up timepoint label of the comparison pair</t>
+          <t>Global Urban Heat Vulnerability Index (GUHVI) class, from 1 (least vulnerable) to 5 (most vulnerable)</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>t1</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr"/>
-      <c r="E99" t="inlineStr"/>
+          <t>urban_heat_guhvi_class</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>class 1-5</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point, grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: urban heat vulnerability</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Indicator value at the baseline timepoint</t>
+          <t>Percentage of population in Global Urban Heat Vulnerability Index (GUHVI) class 5, the most vulnerable class</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>value_t0</t>
-        </is>
-      </c>
-      <c r="D100" t="inlineStr"/>
-      <c r="E100" t="inlineStr"/>
+          <t>pct_urban_heat_guhvi_class_5_most_vulnerable</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>percent</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>percentage</t>
+        </is>
+      </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>grid, city, custom areas</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: composite indices</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Indicator value at the follow-up timepoint</t>
+          <t>Composite index score (Mazziotta-Pareto Index): the mean of the normalised indicators (100 = reference) less a penalty for how unbalanced they are</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>value_t1</t>
-        </is>
-      </c>
-      <c r="D101" t="inlineStr"/>
-      <c r="E101" t="inlineStr"/>
+          <t>sp_index_[index]</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>index (100 = reference)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: composite indices</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Change metric: 'pp_change' (percentage point change; used for bounded percentage indicators), 'diff' (absolute difference) or 'pct_change' (relative change, %, masked where the baseline is zero)</t>
+          <t>Domain score: the mean of the domain's normalised indicators (100 = reference) less a penalty for how unbalanced they are</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>metric</t>
-        </is>
-      </c>
-      <c r="D102" t="inlineStr"/>
-      <c r="E102" t="inlineStr"/>
+          <t>sp_index_[index]__[domain]</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>index (100 = reference)</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: composite indices</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Change in the indicator between t0 and t1, as per the change metric</t>
+          <t>Indicator score: the normalised value of one of the index's indicators (100 = reference), oriented so that higher is better; written once, however many domains it counts towards</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>change</t>
-        </is>
-      </c>
-      <c r="D103" t="inlineStr"/>
-      <c r="E103" t="inlineStr"/>
+          <t>sp_index_[index]__[indicator]</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>index (100 = reference)</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: composite indices</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Whether a policy review checklist was configured and scored for this timepoint</t>
+          <t>Mean level of the normalised indicators or domain scores, before the penalty</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>assessed</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr"/>
-      <c r="E104" t="inlineStr"/>
+          <t>sp_index_[index]_mean</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>index (100 = reference)</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: composite indices</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Policy review checklist version</t>
+          <t>Penalty for imbalance (standard deviation multiplied by the coefficient of variation)</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>checklist_version</t>
-        </is>
-      </c>
-      <c r="D105" t="inlineStr"/>
-      <c r="E105" t="inlineStr"/>
+          <t>sp_index_[index]_penalty</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>index (100 = reference)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: composite indices</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Count of policies identified as present in the policy review</t>
+          <t>Number of indicators contributing</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>presence_numerator</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr"/>
-      <c r="E106" t="inlineStr"/>
+          <t>sp_index_[index]_n</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>count</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>sample point</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: composite indices</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Number of policies assessed for presence in the policy review</t>
+          <t>Average across sample points of the composite index score</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>presence_denominator</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr"/>
-      <c r="E107" t="inlineStr"/>
+          <t>index_[index]</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>index (100 = reference)</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: composite indices</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Policy presence score (%)</t>
+          <t>Average across sample points of the domain score</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>presence_pct</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr"/>
-      <c r="E108" t="inlineStr"/>
+          <t>index_[index]__[domain]</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>index (100 = reference)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: composite indices</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Sum of policy quality scores in the policy review</t>
+          <t>Average across sample points of the indicator score</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>quality_numerator</t>
-        </is>
-      </c>
-      <c r="D109" t="inlineStr"/>
-      <c r="E109" t="inlineStr"/>
+          <t>index_[index]__[indicator]</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>index (100 = reference)</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>grid, custom areas</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Longitudinal series outputs</t>
+          <t>Indicator estimates: composite indices</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Maximum possible sum of policy quality scores in the policy review</t>
+          <t>Average across sample points of the composite index score (population weighted)</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>quality_denominator</t>
-        </is>
-      </c>
-      <c r="D110" t="inlineStr"/>
-      <c r="E110" t="inlineStr"/>
+          <t>pop_index_[index]</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>index (100 = reference)</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>mean</t>
+        </is>
+      </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>longitudinal series</t>
+          <t>city, custom areas</t>
         </is>
       </c>
     </row>
@@ -3616,17 +3760,449 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Policy quality score (%)</t>
+          <t>Timepoint label of the observation (e.g. year)</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>quality_pct</t>
+          <t>timepoint</t>
         </is>
       </c>
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr"/>
       <c r="F111" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Output variable name of the indicator observed (see the indicator entries of this data dictionary)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>indicator</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr"/>
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Value of the indicator at this timepoint for this unit</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr"/>
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Custom area identifier (area panels)</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>area_id</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr"/>
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Unit identifier (generic panels)</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>unit_id</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr"/>
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Baseline timepoint label of the comparison pair</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>t0</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr"/>
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Follow-up timepoint label of the comparison pair</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>t1</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr"/>
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Indicator value at the baseline timepoint</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>value_t0</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr"/>
+      <c r="E118" t="inlineStr"/>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Indicator value at the follow-up timepoint</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>value_t1</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr"/>
+      <c r="E119" t="inlineStr"/>
+      <c r="F119" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Change metric: 'pp_change' (percentage point change; used for bounded percentage indicators), 'diff' (absolute difference) or 'pct_change' (relative change, %, masked where the baseline is zero)</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr"/>
+      <c r="E120" t="inlineStr"/>
+      <c r="F120" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Change in the indicator between t0 and t1, as per the change metric</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>change</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr"/>
+      <c r="E121" t="inlineStr"/>
+      <c r="F121" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Whether a policy review checklist was configured and scored for this timepoint</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>assessed</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr"/>
+      <c r="E122" t="inlineStr"/>
+      <c r="F122" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Policy review checklist version</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>checklist_version</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr"/>
+      <c r="E123" t="inlineStr"/>
+      <c r="F123" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Count of policies identified as present in the policy review</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>presence_numerator</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr"/>
+      <c r="E124" t="inlineStr"/>
+      <c r="F124" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Number of policies assessed for presence in the policy review</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>presence_denominator</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr"/>
+      <c r="E125" t="inlineStr"/>
+      <c r="F125" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Policy presence score (%)</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>presence_pct</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr"/>
+      <c r="E126" t="inlineStr"/>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Sum of policy quality scores in the policy review</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>quality_numerator</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr"/>
+      <c r="E127" t="inlineStr"/>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Maximum possible sum of policy quality scores in the policy review</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>quality_denominator</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr"/>
+      <c r="E128" t="inlineStr"/>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>longitudinal series</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Longitudinal series outputs</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Policy quality score (%)</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>quality_pct</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr"/>
+      <c r="E129" t="inlineStr"/>
+      <c r="F129" t="inlineStr">
         <is>
           <t>longitudinal series</t>
         </is>

</xml_diff>